<commit_message>
update to kow ad
</commit_message>
<xml_diff>
--- a/app/chemalize/episuite/reference_data/Appendix_A_KOWWIN.xlsx
+++ b/app/chemalize/episuite/reference_data/Appendix_A_KOWWIN.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Karez/Nextcloud/QsarLab/Epi_suite/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Karez/Repo/Chemalize/app/chemalize/episuite/reference_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B686FB6-4F48-A54B-BEE1-041090FF532B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29E8B2F0-5A9B-7D42-B7CD-BB775E7A9DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12280" yWindow="6500" windowWidth="27440" windowHeight="16240" xr2:uid="{C34931C6-A040-0745-A0F6-F869DC7D285D}"/>
+    <workbookView xWindow="7120" yWindow="4800" windowWidth="27440" windowHeight="16240" xr2:uid="{C34931C6-A040-0745-A0F6-F869DC7D285D}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="883" uniqueCount="789">
   <si>
     <t>Fragment Descriptor</t>
   </si>
@@ -2329,6 +2329,102 @@
   </si>
   <si>
     <t>aliph-CH=N-O-carbon(aliphat) [iminoxy] cor</t>
+  </si>
+  <si>
+    <t>1.4148</t>
+  </si>
+  <si>
+    <t>1.3369</t>
+  </si>
+  <si>
+    <t>1.2800</t>
+  </si>
+  <si>
+    <t>1.7110</t>
+  </si>
+  <si>
+    <t>1.1930</t>
+  </si>
+  <si>
+    <t>1.3548</t>
+  </si>
+  <si>
+    <t>2.2489</t>
+  </si>
+  <si>
+    <t>1.3536</t>
+  </si>
+  <si>
+    <t>1.4790</t>
+  </si>
+  <si>
+    <t>1.2</t>
+  </si>
+  <si>
+    <t>2.6156</t>
+  </si>
+  <si>
+    <t>1.4227</t>
+  </si>
+  <si>
+    <t>1.2295</t>
+  </si>
+  <si>
+    <t>1.7838</t>
+  </si>
+  <si>
+    <t>1.2556</t>
+  </si>
+  <si>
+    <t>1.5505</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1.3226</t>
+  </si>
+  <si>
+    <t>1.8</t>
+  </si>
+  <si>
+    <t>1.43</t>
+  </si>
+  <si>
+    <t>1.55</t>
+  </si>
+  <si>
+    <t>1.5</t>
+  </si>
+  <si>
+    <t>1.25</t>
+  </si>
+  <si>
+    <t>1.35</t>
+  </si>
+  <si>
+    <t>1.95</t>
+  </si>
+  <si>
+    <t>1.6</t>
+  </si>
+  <si>
+    <t>2.75</t>
+  </si>
+  <si>
+    <t>1.9</t>
+  </si>
+  <si>
+    <t>1.42</t>
+  </si>
+  <si>
+    <t>1.3</t>
+  </si>
+  <si>
+    <t>2.5</t>
+  </si>
+  <si>
+    <t>1.6450</t>
+  </si>
+  <si>
+    <t>2.4000</t>
   </si>
 </sst>
 </file>
@@ -2391,8 +2487,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hiperłącze" xfId="1" builtinId="8"/>
-    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2408,9 +2504,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motyw pakietu Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Pakiet Office">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2448,7 +2544,7 @@
         <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Pakiet Office">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
@@ -2554,7 +2650,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Pakiet Office">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2931,8 +3027,8 @@
       <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="2">
-        <v>821067</v>
+      <c r="B11" s="2" t="s">
+        <v>757</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -4251,8 +4347,8 @@
       <c r="A77" t="s">
         <v>155</v>
       </c>
-      <c r="B77" s="2">
-        <v>536544</v>
+      <c r="B77" s="2" t="s">
+        <v>758</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -4931,8 +5027,8 @@
       <c r="A111" t="s">
         <v>220</v>
       </c>
-      <c r="B111" s="2">
-        <v>328720</v>
+      <c r="B111" s="2" t="s">
+        <v>759</v>
       </c>
       <c r="C111">
         <v>1</v>
@@ -5051,8 +5147,8 @@
       <c r="A117" t="s">
         <v>231</v>
       </c>
-      <c r="B117" s="2">
-        <v>1902915</v>
+      <c r="B117" s="2" t="s">
+        <v>760</v>
       </c>
       <c r="C117">
         <v>1</v>
@@ -5931,8 +6027,8 @@
       <c r="A162" t="s">
         <v>310</v>
       </c>
-      <c r="B162" s="2">
-        <v>10959</v>
+      <c r="B162" s="2" t="s">
+        <v>761</v>
       </c>
       <c r="C162">
         <v>1</v>
@@ -6131,8 +6227,8 @@
       <c r="A172" t="s">
         <v>329</v>
       </c>
-      <c r="B172" s="2">
-        <v>601921</v>
+      <c r="B172" s="2" t="s">
+        <v>762</v>
       </c>
       <c r="C172">
         <v>1</v>
@@ -6651,8 +6747,8 @@
       <c r="A198" t="s">
         <v>380</v>
       </c>
-      <c r="B198" s="2">
-        <v>215162</v>
+      <c r="B198" s="2" t="s">
+        <v>763</v>
       </c>
       <c r="C198">
         <v>1</v>
@@ -6731,8 +6827,8 @@
       <c r="A202" t="s">
         <v>387</v>
       </c>
-      <c r="B202" s="2">
-        <v>597538</v>
+      <c r="B202" s="2" t="s">
+        <v>764</v>
       </c>
       <c r="C202">
         <v>1</v>
@@ -6791,8 +6887,8 @@
       <c r="A205" t="s">
         <v>392</v>
       </c>
-      <c r="B205" s="2">
-        <v>1055553</v>
+      <c r="B205" s="2" t="s">
+        <v>765</v>
       </c>
       <c r="C205">
         <v>1</v>
@@ -6891,8 +6987,8 @@
       <c r="A210" t="s">
         <v>401</v>
       </c>
-      <c r="B210" s="2">
-        <v>36526</v>
+      <c r="B210" s="2" t="s">
+        <v>766</v>
       </c>
       <c r="C210">
         <v>1</v>
@@ -7011,8 +7107,8 @@
       <c r="A216" t="s">
         <v>412</v>
       </c>
-      <c r="B216" s="2">
-        <v>1554505</v>
+      <c r="B216" s="2" t="s">
+        <v>767</v>
       </c>
       <c r="C216">
         <v>1</v>
@@ -7271,8 +7367,8 @@
       <c r="A229" t="s">
         <v>437</v>
       </c>
-      <c r="B229" s="2">
-        <v>849921</v>
+      <c r="B229" s="2" t="s">
+        <v>768</v>
       </c>
       <c r="C229">
         <v>1</v>
@@ -7391,8 +7487,8 @@
       <c r="A235" t="s">
         <v>448</v>
       </c>
-      <c r="B235" s="2">
-        <v>144273</v>
+      <c r="B235" s="2" t="s">
+        <v>769</v>
       </c>
       <c r="C235">
         <v>1</v>
@@ -7611,8 +7707,8 @@
       <c r="A246" t="s">
         <v>469</v>
       </c>
-      <c r="B246" s="2">
-        <v>2168812</v>
+      <c r="B246" s="2" t="s">
+        <v>770</v>
       </c>
       <c r="C246">
         <v>1</v>
@@ -7891,8 +7987,8 @@
       <c r="A260" t="s">
         <v>496</v>
       </c>
-      <c r="B260" s="2">
-        <v>239601</v>
+      <c r="B260" s="2" t="s">
+        <v>771</v>
       </c>
       <c r="C260">
         <v>1</v>
@@ -8431,8 +8527,8 @@
       <c r="A287" t="s">
         <v>549</v>
       </c>
-      <c r="B287" s="2">
-        <v>1316701</v>
+      <c r="B287" s="2" t="s">
+        <v>772</v>
       </c>
       <c r="C287">
         <v>1</v>
@@ -8891,8 +8987,8 @@
       <c r="A310" t="s">
         <v>584</v>
       </c>
-      <c r="B310" s="2">
-        <v>484314</v>
+      <c r="B310" s="2" t="s">
+        <v>773</v>
       </c>
       <c r="C310">
         <v>1</v>
@@ -8971,8 +9067,8 @@
       <c r="A314" t="s">
         <v>591</v>
       </c>
-      <c r="B314" s="2">
-        <v>2227981</v>
+      <c r="B314" s="2" t="s">
+        <v>774</v>
       </c>
       <c r="C314">
         <v>1</v>
@@ -9011,8 +9107,8 @@
       <c r="A316" t="s">
         <v>593</v>
       </c>
-      <c r="B316" s="2">
-        <v>876584</v>
+      <c r="B316" s="2" t="s">
+        <v>775</v>
       </c>
       <c r="C316">
         <v>1</v>
@@ -9151,8 +9247,8 @@
       <c r="A323" t="s">
         <v>604</v>
       </c>
-      <c r="B323" s="2">
-        <v>36526</v>
+      <c r="B323" s="2" t="s">
+        <v>766</v>
       </c>
       <c r="C323">
         <v>1</v>
@@ -9171,8 +9267,8 @@
       <c r="A324" t="s">
         <v>605</v>
       </c>
-      <c r="B324" s="2">
-        <v>1314875</v>
+      <c r="B324" s="2" t="s">
+        <v>776</v>
       </c>
       <c r="C324">
         <v>1</v>
@@ -9371,8 +9467,8 @@
       <c r="A334" t="s">
         <v>616</v>
       </c>
-      <c r="B334" s="2">
-        <v>1132254</v>
+      <c r="B334" s="2" t="s">
+        <v>777</v>
       </c>
       <c r="C334">
         <v>1</v>
@@ -9654,8 +9750,8 @@
       <c r="A348" t="s">
         <v>635</v>
       </c>
-      <c r="B348" s="2">
-        <v>219148</v>
+      <c r="B348" s="2" t="s">
+        <v>778</v>
       </c>
       <c r="C348">
         <v>1</v>
@@ -9694,8 +9790,8 @@
       <c r="A350" t="s">
         <v>638</v>
       </c>
-      <c r="B350" s="2">
-        <v>219148</v>
+      <c r="B350" s="2" t="s">
+        <v>778</v>
       </c>
       <c r="C350">
         <v>1</v>
@@ -9714,8 +9810,8 @@
       <c r="A351" t="s">
         <v>639</v>
       </c>
-      <c r="B351" s="2">
-        <v>36526</v>
+      <c r="B351" s="2" t="s">
+        <v>766</v>
       </c>
       <c r="C351">
         <v>1</v>
@@ -9934,8 +10030,8 @@
       <c r="A362" t="s">
         <v>653</v>
       </c>
-      <c r="B362" s="2">
-        <v>584390</v>
+      <c r="B362" s="2" t="s">
+        <v>779</v>
       </c>
       <c r="C362">
         <v>1</v>
@@ -9994,8 +10090,8 @@
       <c r="A365" t="s">
         <v>657</v>
       </c>
-      <c r="B365" s="2">
-        <v>2775845</v>
+      <c r="B365" s="2" t="s">
+        <v>780</v>
       </c>
       <c r="C365">
         <v>1</v>
@@ -10154,8 +10250,8 @@
       <c r="A373" t="s">
         <v>668</v>
       </c>
-      <c r="B373" s="2">
-        <v>1497496</v>
+      <c r="B373" s="2" t="s">
+        <v>781</v>
       </c>
       <c r="C373">
         <v>1</v>
@@ -10374,8 +10470,8 @@
       <c r="A384" t="s">
         <v>684</v>
       </c>
-      <c r="B384" s="2">
-        <v>36526</v>
+      <c r="B384" s="2" t="s">
+        <v>766</v>
       </c>
       <c r="C384">
         <v>1</v>
@@ -10754,8 +10850,8 @@
       <c r="A403" t="s">
         <v>707</v>
       </c>
-      <c r="B403" s="2">
-        <v>2045391</v>
+      <c r="B403" s="2" t="s">
+        <v>782</v>
       </c>
       <c r="C403">
         <v>1</v>
@@ -10914,8 +11010,8 @@
       <c r="A411" t="s">
         <v>721</v>
       </c>
-      <c r="B411" s="2">
-        <v>2593224</v>
+      <c r="B411" s="2" t="s">
+        <v>783</v>
       </c>
       <c r="C411">
         <v>1</v>
@@ -10954,8 +11050,8 @@
       <c r="A413" t="s">
         <v>723</v>
       </c>
-      <c r="B413" s="2">
-        <v>840060</v>
+      <c r="B413" s="2" t="s">
+        <v>784</v>
       </c>
       <c r="C413">
         <v>1</v>
@@ -11114,8 +11210,8 @@
       <c r="A421" t="s">
         <v>732</v>
       </c>
-      <c r="B421" s="2">
-        <v>401769</v>
+      <c r="B421" s="2" t="s">
+        <v>785</v>
       </c>
       <c r="C421">
         <v>1</v>
@@ -11174,8 +11270,8 @@
       <c r="A424" t="s">
         <v>735</v>
       </c>
-      <c r="B424" s="2">
-        <v>1132285</v>
+      <c r="B424" s="2" t="s">
+        <v>786</v>
       </c>
       <c r="C424">
         <v>1</v>
@@ -11354,8 +11450,8 @@
       <c r="A433" t="s">
         <v>748</v>
       </c>
-      <c r="B433" s="2">
-        <v>1661856</v>
+      <c r="B433" s="2" t="s">
+        <v>787</v>
       </c>
       <c r="C433">
         <v>1</v>
@@ -11394,8 +11490,8 @@
       <c r="A435" t="s">
         <v>750</v>
       </c>
-      <c r="B435" s="2">
-        <v>767042</v>
+      <c r="B435" s="2" t="s">
+        <v>788</v>
       </c>
       <c r="C435">
         <v>1</v>

</xml_diff>